<commit_message>
week 4 material fix
</commit_message>
<xml_diff>
--- a/material/Week3-Objectives/SkillsCheckTeamAnswers.xlsx
+++ b/material/Week3-Objectives/SkillsCheckTeamAnswers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailmissouri-my.sharepoint.com/personal/btdhd_umsystem_edu/Documents/Desktop/NATR_8001_DecisionAnalysis_Fall25_Mizzou/material/Week3-Objectives/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27D04C99-DE25-4B11-BC2A-F94835561C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{27D04C99-DE25-4B11-BC2A-F94835561C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16D6955A-85C3-438C-B10E-1635290F94A0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33EB1A41-E2EE-475D-8F0F-7978F121B234}"/>
+    <workbookView xWindow="9510" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{33EB1A41-E2EE-475D-8F0F-7978F121B234}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t>Team 1</t>
   </si>
@@ -60,6 +60,90 @@
   </si>
   <si>
     <t>Strategic objectives</t>
+  </si>
+  <si>
+    <t>Maximize lizard persistence</t>
+  </si>
+  <si>
+    <t>Minimize cost</t>
+  </si>
+  <si>
+    <t>reduce road crossing events</t>
+  </si>
+  <si>
+    <t>Maximize lizard population</t>
+  </si>
+  <si>
+    <t>Maximize survival</t>
+  </si>
+  <si>
+    <t>Maximize habitat</t>
+  </si>
+  <si>
+    <t>Minimize road use</t>
+  </si>
+  <si>
+    <t>Increase lizard persistence</t>
+  </si>
+  <si>
+    <t>Maximize visitor experience</t>
+  </si>
+  <si>
+    <t>Increase reproduction</t>
+  </si>
+  <si>
+    <t>Decrese mortality</t>
+  </si>
+  <si>
+    <t>Increase habitat</t>
+  </si>
+  <si>
+    <t>Increase acesss</t>
+  </si>
+  <si>
+    <t>Maximize recreation opportunities</t>
+  </si>
+  <si>
+    <t>Increase survival</t>
+  </si>
+  <si>
+    <t>Minmize disturbance to visitors</t>
+  </si>
+  <si>
+    <t>Increase public recreation</t>
+  </si>
+  <si>
+    <t>Decrease cost</t>
+  </si>
+  <si>
+    <t>Minimize car deaths</t>
+  </si>
+  <si>
+    <t>Maximize birding opportunities</t>
+  </si>
+  <si>
+    <t>Team 5</t>
+  </si>
+  <si>
+    <t>Increase recreation accessibility</t>
+  </si>
+  <si>
+    <t>Decrease conflict</t>
+  </si>
+  <si>
+    <t>Respect birding folks</t>
+  </si>
+  <si>
+    <t>Increase habitat connectivity</t>
+  </si>
+  <si>
+    <t>Minimize effects on recreation</t>
+  </si>
+  <si>
+    <t>Increase burn effectiveness</t>
+  </si>
+  <si>
+    <t>increase action efficiency</t>
   </si>
 </sst>
 </file>
@@ -431,14 +515,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D13CC3D-8438-4D27-A22E-76676FF5D720}">
-  <dimension ref="A2:E22"/>
+  <dimension ref="A2:F23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -451,24 +539,150 @@
       <c r="E2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>